<commit_message>
correção markov-switching uni switching var 2020
</commit_message>
<xml_diff>
--- a/ox/variaveis_previsao.xlsx
+++ b/ox/variaveis_previsao.xlsx
@@ -64704,7 +64704,7 @@
         <v>-0.034762643876947594</v>
       </c>
       <c r="X206" t="n">
-        <v>-0.033195761382440174</v>
+        <v>-0.056294071154285627</v>
       </c>
       <c r="Y206" t="n">
         <v>-0.033195761382440174</v>
@@ -65011,7 +65011,7 @@
         <v>-0.058720366188525205</v>
       </c>
       <c r="X207" t="n">
-        <v>-0.058446250731468787</v>
+        <v>-0.060842729538109916</v>
       </c>
       <c r="Y207" t="n">
         <v>-0.058446250731468787</v>
@@ -65318,7 +65318,7 @@
         <v>0.019021752601873325</v>
       </c>
       <c r="X208" t="n">
-        <v>0.019424137965712365</v>
+        <v>0.020462409309620323</v>
       </c>
       <c r="Y208" t="n">
         <v>0.019424137965712365</v>
@@ -65625,7 +65625,7 @@
         <v>0.038922703160038596</v>
       </c>
       <c r="X209" t="n">
-        <v>0.039058577172908712</v>
+        <v>0.041270829650434937</v>
       </c>
       <c r="Y209" t="n">
         <v>0.039058577172908712</v>
@@ -65932,7 +65932,7 @@
         <v>-0.0029745206844050669</v>
       </c>
       <c r="X210" t="n">
-        <v>-0.0048874063551694385</v>
+        <v>-0.017745878635717353</v>
       </c>
       <c r="Y210" t="n">
         <v>-0.0048874063551694385</v>
@@ -66239,7 +66239,7 @@
         <v>0.00655228948957214</v>
       </c>
       <c r="X211" t="n">
-        <v>0.0062547598779566071</v>
+        <v>0.010580444237972947</v>
       </c>
       <c r="Y211" t="n">
         <v>0.0062547598779566071</v>
@@ -66546,7 +66546,7 @@
         <v>0.006415354400758526</v>
       </c>
       <c r="X212" t="n">
-        <v>0.0044044106290735408</v>
+        <v>0.0070278576731419209</v>
       </c>
       <c r="Y212" t="n">
         <v>0.0044044106290735408</v>
@@ -66853,7 +66853,7 @@
         <v>0.012401614851858726</v>
       </c>
       <c r="X213" t="n">
-        <v>0.013227803357760727</v>
+        <v>0.027823999757744085</v>
       </c>
       <c r="Y213" t="n">
         <v>0.013227803357760727</v>
@@ -67160,7 +67160,7 @@
         <v>0.033243167078601636</v>
       </c>
       <c r="X214" t="n">
-        <v>0.031490538643956942</v>
+        <v>0.022804642701206537</v>
       </c>
       <c r="Y214" t="n">
         <v>0.031490538643956942</v>
@@ -67467,7 +67467,7 @@
         <v>0.019410555739571511</v>
       </c>
       <c r="X215" t="n">
-        <v>0.019539542244047938</v>
+        <v>0.020355070610711779</v>
       </c>
       <c r="Y215" t="n">
         <v>0.019539542244047938</v>
@@ -67774,7 +67774,7 @@
         <v>-0.0055923693980736598</v>
       </c>
       <c r="X216" t="n">
-        <v>-0.004996848893835869</v>
+        <v>0.0074383257068174509</v>
       </c>
       <c r="Y216" t="n">
         <v>-0.004996848893835869</v>
@@ -68081,7 +68081,7 @@
         <v>0.067679103865961654</v>
       </c>
       <c r="X217" t="n">
-        <v>0.066880230602769375</v>
+        <v>0.0546491781517459</v>
       </c>
       <c r="Y217" t="n">
         <v>0.066880230602769375</v>

</xml_diff>